<commit_message>
Curva S actualizada 2026-07-17 17:11 Chile
</commit_message>
<xml_diff>
--- a/data/50001515 - CLIENTE POR DEFINIR B.xlsx
+++ b/data/50001515 - CLIENTE POR DEFINIR B.xlsx
@@ -2320,7 +2320,7 @@
         <v>46114.5135508449</v>
       </c>
       <c r="D18" s="5">
-        <v>46114.51356479166</v>
+        <v>46220.87441708334</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>76</v>
@@ -2694,7 +2694,7 @@
         <v>46155.829147384255</v>
       </c>
       <c r="D24" s="5">
-        <v>46155.829164849536</v>
+        <v>46220.86329395833</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>94</v>

</xml_diff>